<commit_message>
Eliminacion de código de graficos innecesario
se eliminan codigos de graficos generados por fases,
</commit_message>
<xml_diff>
--- a/documentacion/Plan_Tesis_2026_Gantt_Seguimiento.xlsx
+++ b/documentacion/Plan_Tesis_2026_Gantt_Seguimiento.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\UPMH - Maestría en Inteligencia Artificial\Sexto cuatrimestre\Tesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\tesis\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF14E0C-D21C-4B61-9CFB-BCDD7B596B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388ADF95-472C-455E-92A6-F9B8641C554E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma Tesis (V2)" sheetId="2" r:id="rId1"/>
@@ -895,20 +895,20 @@
     <tabColor rgb="FF00B050"/>
   </sheetPr>
   <dimension ref="A1:AD20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.42578125" customWidth="1"/>
-    <col min="4" max="5" width="11.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.44140625" customWidth="1"/>
+    <col min="4" max="5" width="11.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" style="4" customWidth="1"/>
     <col min="7" max="7" width="11" style="4" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="17" width="4.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="17" width="4.88671875" customWidth="1"/>
     <col min="18" max="30" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -1028,7 +1028,7 @@
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
     </row>
-    <row r="3" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="M5" s="6"/>
     </row>
-    <row r="6" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="N6" s="6"/>
     </row>
-    <row r="7" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="O7" s="6"/>
     </row>
-    <row r="8" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -1191,7 +1191,7 @@
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7">
         <v>8</v>
       </c>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
         <v>9</v>
       </c>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="Q10" s="6"/>
     </row>
-    <row r="11" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7">
         <v>10</v>
       </c>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="R11" s="6"/>
     </row>
-    <row r="12" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
         <v>11</v>
       </c>
@@ -1292,14 +1292,14 @@
         <v>1</v>
       </c>
       <c r="G12" s="10">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H12" t="s">
         <v>85</v>
       </c>
-      <c r="S12" s="11"/>
-    </row>
-    <row r="13" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S12" s="6"/>
+    </row>
+    <row r="13" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="7">
         <v>11</v>
       </c>
@@ -1319,15 +1319,15 @@
         <v>3</v>
       </c>
       <c r="G13" s="10">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H13" t="s">
         <v>50</v>
       </c>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
-    </row>
-    <row r="14" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+    </row>
+    <row r="14" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7">
         <v>12</v>
       </c>
@@ -1347,14 +1347,14 @@
         <v>1</v>
       </c>
       <c r="G14" s="10">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H14" t="s">
         <v>50</v>
       </c>
-      <c r="V14" s="5"/>
-    </row>
-    <row r="15" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="V14" s="11"/>
+    </row>
+    <row r="15" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="7">
         <v>13</v>
       </c>
@@ -1382,7 +1382,7 @@
       <c r="W15" s="5"/>
       <c r="X15" s="5"/>
     </row>
-    <row r="16" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>14</v>
       </c>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="Y16" s="5"/>
     </row>
-    <row r="17" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
         <v>15</v>
       </c>
@@ -1437,7 +1437,7 @@
       <c r="Z17" s="5"/>
       <c r="AA17" s="5"/>
     </row>
-    <row r="18" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7">
         <v>16</v>
       </c>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="AB18" s="5"/>
     </row>
-    <row r="19" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7">
         <v>17</v>
       </c>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="AC19" s="5"/>
     </row>
-    <row r="20" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7">
         <v>18</v>
       </c>
@@ -1532,20 +1532,20 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:AV23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" style="4" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="17" width="4.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="17" width="4.88671875" customWidth="1"/>
     <col min="18" max="48" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1719,7 +1719,7 @@
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
     </row>
-    <row r="3" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1775,7 +1775,7 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1804,7 +1804,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
     </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1832,7 +1832,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
     </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1860,7 +1860,7 @@
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
     </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1888,7 +1888,7 @@
       <c r="V8" s="6"/>
       <c r="W8" s="6"/>
     </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1916,7 +1916,7 @@
       <c r="X9" s="6"/>
       <c r="Y9" s="6"/>
     </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1944,7 +1944,7 @@
       <c r="Z10" s="5"/>
       <c r="AA10" s="5"/>
     </row>
-    <row r="11" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="AB11" s="5"/>
     </row>
-    <row r="12" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2000,7 +2000,7 @@
       <c r="AD12" s="5"/>
       <c r="AE12" s="5"/>
     </row>
-    <row r="13" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2028,7 +2028,7 @@
       <c r="AF13" s="5"/>
       <c r="AG13" s="5"/>
     </row>
-    <row r="14" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="AH14" s="5"/>
     </row>
-    <row r="15" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2083,7 +2083,7 @@
       <c r="AI15" s="5"/>
       <c r="AJ15" s="5"/>
     </row>
-    <row r="16" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2111,7 +2111,7 @@
       <c r="AK16" s="5"/>
       <c r="AL16" s="5"/>
     </row>
-    <row r="17" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2139,7 +2139,7 @@
       <c r="AM17" s="5"/>
       <c r="AN17" s="5"/>
     </row>
-    <row r="18" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2167,7 +2167,7 @@
       <c r="AO18" s="5"/>
       <c r="AP18" s="5"/>
     </row>
-    <row r="19" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="AQ19" s="5"/>
     </row>
-    <row r="20" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2222,7 +2222,7 @@
       <c r="AR20" s="5"/>
       <c r="AS20" s="5"/>
     </row>
-    <row r="21" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2250,7 +2250,7 @@
       <c r="AT21" s="5"/>
       <c r="AU21" s="5"/>
     </row>
-    <row r="22" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="AV22" s="5"/>
     </row>
-    <row r="23" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:48" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
cambios a la investigacion 24ago2026
</commit_message>
<xml_diff>
--- a/documentacion/Plan_Tesis_2026_Gantt_Seguimiento.xlsx
+++ b/documentacion/Plan_Tesis_2026_Gantt_Seguimiento.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\tesis\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F47E95C-8714-41C0-B8AC-26A50C4F7FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A3939C-9065-4939-8C23-C4DCC07B30CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="68">
   <si>
     <t>ID</t>
   </si>
@@ -209,6 +209,21 @@
   </si>
   <si>
     <t>Entrenar modelos</t>
+  </si>
+  <si>
+    <t>AGOSTO</t>
+  </si>
+  <si>
+    <t>JULIO</t>
+  </si>
+  <si>
+    <t>JUNIO</t>
+  </si>
+  <si>
+    <t>MAYO</t>
+  </si>
+  <si>
+    <t>ABRIL</t>
   </si>
 </sst>
 </file>
@@ -236,7 +251,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -262,7 +277,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -294,7 +315,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -321,6 +342,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -377,8 +402,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10128EF7-60C2-43B4-A723-CD25FC0BA309}" name="Tabla13" displayName="Tabla13" ref="A1:AD20" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:AD20" xr:uid="{FEA64A45-B8C0-40A5-9558-FE32A9E3005A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{10128EF7-60C2-43B4-A723-CD25FC0BA309}" name="Tabla13" displayName="Tabla13" ref="A2:AD39" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A2:AD39" xr:uid="{FEA64A45-B8C0-40A5-9558-FE32A9E3005A}"/>
   <tableColumns count="30">
     <tableColumn id="1" xr3:uid="{3B51200C-56FE-492D-BA6F-F51AA338B09C}" name="ID"/>
     <tableColumn id="2" xr3:uid="{4E22F30B-C7CA-48A9-AFAD-148B9046592C}" name="Fase"/>
@@ -703,12 +728,12 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:AD20"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.44140625" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.77734375" customWidth="1"/>
     <col min="4" max="5" width="11.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.109375" style="4" customWidth="1"/>
     <col min="7" max="7" width="11" style="4" customWidth="1"/>
@@ -717,144 +742,148 @@
     <col min="18" max="30" width="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="I1" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="13"/>
+    </row>
+    <row r="2" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="9">
-        <v>46132</v>
-      </c>
-      <c r="E2" s="9">
-        <v>46145</v>
-      </c>
-      <c r="F2" s="10">
-        <v>2</v>
-      </c>
-      <c r="G2" s="10">
-        <v>100</v>
-      </c>
-      <c r="H2" t="s">
-        <v>51</v>
-      </c>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
     </row>
     <row r="3" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D3" s="9">
-        <v>46146</v>
+        <v>46132</v>
       </c>
       <c r="E3" s="9">
-        <v>46152</v>
+        <v>46145</v>
       </c>
       <c r="F3" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="10">
         <v>100</v>
@@ -862,50 +891,35 @@
       <c r="H3" t="s">
         <v>51</v>
       </c>
-      <c r="K3" s="6"/>
-    </row>
-    <row r="4" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7">
-        <v>3</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="9">
-        <v>46153</v>
-      </c>
-      <c r="E4" s="9">
-        <v>46159</v>
-      </c>
-      <c r="F4" s="10">
-        <v>1</v>
-      </c>
-      <c r="G4" s="10">
-        <v>100</v>
-      </c>
-      <c r="H4" t="s">
-        <v>51</v>
-      </c>
-      <c r="L4" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="4" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
     </row>
     <row r="5" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D5" s="9">
-        <v>46160</v>
+        <v>46146</v>
       </c>
       <c r="E5" s="9">
-        <v>46166</v>
+        <v>46152</v>
       </c>
       <c r="F5" s="10">
         <v>1</v>
@@ -916,159 +930,107 @@
       <c r="H5" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7">
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="K6" s="11"/>
+    </row>
+    <row r="7" spans="1:30" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="9">
+        <v>46153</v>
+      </c>
+      <c r="E7" s="9">
+        <v>46159</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10">
+        <v>100</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="6"/>
+    </row>
+    <row r="8" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="L8" s="11"/>
+    </row>
+    <row r="9" spans="1:30" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>4</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="9">
+        <v>46160</v>
+      </c>
+      <c r="E9" s="9">
+        <v>46166</v>
+      </c>
+      <c r="F9" s="10">
+        <v>1</v>
+      </c>
+      <c r="G9" s="10">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="M9" s="6"/>
+    </row>
+    <row r="10" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="M10" s="11"/>
+    </row>
+    <row r="11" spans="1:30" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D11" s="9">
         <v>46167</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E11" s="9">
         <v>46170</v>
-      </c>
-      <c r="F6" s="10">
-        <v>1</v>
-      </c>
-      <c r="G6" s="10">
-        <v>100</v>
-      </c>
-      <c r="H6" t="s">
-        <v>51</v>
-      </c>
-      <c r="N6" s="6"/>
-    </row>
-    <row r="7" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="9">
-        <v>46171</v>
-      </c>
-      <c r="E7" s="9">
-        <v>46173</v>
-      </c>
-      <c r="F7" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="G7" s="10">
-        <v>100</v>
-      </c>
-      <c r="H7" t="s">
-        <v>51</v>
-      </c>
-      <c r="O7" s="6"/>
-    </row>
-    <row r="8" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="7">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="9">
-        <v>46174</v>
-      </c>
-      <c r="E8" s="9">
-        <v>46188</v>
-      </c>
-      <c r="F8" s="10">
-        <v>2</v>
-      </c>
-      <c r="G8" s="10">
-        <v>100</v>
-      </c>
-      <c r="H8" t="s">
-        <v>51</v>
-      </c>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-    </row>
-    <row r="9" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
-        <v>8</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="9">
-        <v>46189</v>
-      </c>
-      <c r="E9" s="9">
-        <v>46192</v>
-      </c>
-      <c r="F9" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="G9" s="10">
-        <v>100</v>
-      </c>
-      <c r="H9" t="s">
-        <v>51</v>
-      </c>
-      <c r="P9" s="6"/>
-    </row>
-    <row r="10" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="7">
-        <v>9</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="9">
-        <v>46195</v>
-      </c>
-      <c r="E10" s="9">
-        <v>46201</v>
-      </c>
-      <c r="F10" s="10">
-        <v>1</v>
-      </c>
-      <c r="G10" s="10">
-        <v>100</v>
-      </c>
-      <c r="H10" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q10" s="6"/>
-    </row>
-    <row r="11" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="7">
-        <v>10</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="9">
-        <v>46202</v>
-      </c>
-      <c r="E11" s="9">
-        <v>46208</v>
       </c>
       <c r="F11" s="10">
         <v>1</v>
@@ -1079,255 +1041,547 @@
       <c r="H11" t="s">
         <v>51</v>
       </c>
-      <c r="R11" s="6"/>
-    </row>
-    <row r="12" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7">
-        <v>11</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="9">
-        <v>46209</v>
-      </c>
-      <c r="E12" s="9">
-        <v>46213</v>
-      </c>
-      <c r="F12" s="10">
-        <v>1</v>
-      </c>
-      <c r="G12" s="10">
-        <v>100</v>
-      </c>
-      <c r="H12" t="s">
-        <v>52</v>
-      </c>
-      <c r="S12" s="6"/>
+      <c r="N11" s="6"/>
+    </row>
+    <row r="12" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="N12" s="11"/>
     </row>
     <row r="13" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="7">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="D13" s="9">
-        <v>46216</v>
+        <v>46171</v>
       </c>
       <c r="E13" s="9">
-        <v>46229</v>
+        <v>46173</v>
       </c>
       <c r="F13" s="10">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="G13" s="10">
         <v>100</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
-      </c>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-    </row>
-    <row r="14" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="7">
-        <v>12</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D14" s="9">
-        <v>46230</v>
-      </c>
-      <c r="E14" s="9">
-        <v>46236</v>
-      </c>
-      <c r="F14" s="10">
-        <v>1</v>
-      </c>
-      <c r="G14" s="10">
-        <v>100</v>
-      </c>
-      <c r="H14" t="s">
-        <v>32</v>
-      </c>
-      <c r="V14" s="6"/>
+        <v>51</v>
+      </c>
+      <c r="O13" s="6"/>
+    </row>
+    <row r="14" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="O14" s="11"/>
     </row>
     <row r="15" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="7">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D15" s="9">
-        <v>46237</v>
+        <v>46174</v>
       </c>
       <c r="E15" s="9">
-        <v>46250</v>
+        <v>46188</v>
       </c>
       <c r="F15" s="10">
         <v>2</v>
       </c>
       <c r="G15" s="10">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H15" t="s">
-        <v>32</v>
-      </c>
-      <c r="W15" s="6"/>
-      <c r="X15" s="11"/>
-    </row>
-    <row r="16" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="7">
-        <v>14</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="9">
-        <v>46251</v>
-      </c>
-      <c r="E16" s="9">
-        <v>46257</v>
-      </c>
-      <c r="F16" s="10">
-        <v>1</v>
-      </c>
-      <c r="G16" s="10">
-        <v>0</v>
-      </c>
-      <c r="H16" t="s">
-        <v>32</v>
-      </c>
-      <c r="Y16" s="5"/>
-    </row>
-    <row r="17" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+    </row>
+    <row r="16" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+    </row>
+    <row r="17" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="D17" s="9">
-        <v>46258</v>
+        <v>46189</v>
       </c>
       <c r="E17" s="9">
-        <v>46271</v>
+        <v>46192</v>
       </c>
       <c r="F17" s="10">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="G17" s="10">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H17" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z17" s="5"/>
-      <c r="AA17" s="5"/>
-    </row>
-    <row r="18" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="7">
-        <v>16</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="9">
-        <v>46272</v>
-      </c>
-      <c r="E18" s="9">
-        <v>46278</v>
-      </c>
-      <c r="F18" s="10">
-        <v>1</v>
-      </c>
-      <c r="G18" s="10">
-        <v>0</v>
-      </c>
-      <c r="H18" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB18" s="5"/>
-    </row>
-    <row r="19" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+      <c r="P17" s="6"/>
+    </row>
+    <row r="18" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D19" s="9">
-        <v>46279</v>
+        <v>46195</v>
       </c>
       <c r="E19" s="9">
-        <v>46285</v>
+        <v>46201</v>
       </c>
       <c r="F19" s="10">
         <v>1</v>
       </c>
       <c r="G19" s="10">
+        <v>100</v>
+      </c>
+      <c r="H19" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q19" s="6"/>
+    </row>
+    <row r="20" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="7"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="Q20" s="11"/>
+    </row>
+    <row r="21" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
+        <v>10</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="9">
+        <v>46202</v>
+      </c>
+      <c r="E21" s="9">
+        <v>46208</v>
+      </c>
+      <c r="F21" s="10">
+        <v>1</v>
+      </c>
+      <c r="G21" s="10">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>51</v>
+      </c>
+      <c r="R21" s="6"/>
+    </row>
+    <row r="22" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="R22" s="11"/>
+    </row>
+    <row r="23" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7">
+        <v>11</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="9">
+        <v>46209</v>
+      </c>
+      <c r="E23" s="9">
+        <v>46213</v>
+      </c>
+      <c r="F23" s="10">
+        <v>1</v>
+      </c>
+      <c r="G23" s="10">
+        <v>100</v>
+      </c>
+      <c r="H23" t="s">
+        <v>51</v>
+      </c>
+      <c r="S23" s="6"/>
+    </row>
+    <row r="24" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="S24" s="11"/>
+      <c r="T24" s="11"/>
+      <c r="U24" s="11"/>
+    </row>
+    <row r="25" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7">
+        <v>11</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="9">
+        <v>46216</v>
+      </c>
+      <c r="E25" s="9">
+        <v>46229</v>
+      </c>
+      <c r="F25" s="10">
+        <v>3</v>
+      </c>
+      <c r="G25" s="10">
+        <v>100</v>
+      </c>
+      <c r="H25" t="s">
+        <v>51</v>
+      </c>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+    </row>
+    <row r="26" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="7"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="U26" s="11"/>
+      <c r="V26" s="11"/>
+      <c r="W26" s="11"/>
+    </row>
+    <row r="27" spans="1:27" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7">
+        <v>12</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="9">
+        <v>46230</v>
+      </c>
+      <c r="E27" s="9">
+        <v>46236</v>
+      </c>
+      <c r="F27" s="10">
+        <v>1</v>
+      </c>
+      <c r="G27" s="10">
+        <v>100</v>
+      </c>
+      <c r="H27" t="s">
+        <v>51</v>
+      </c>
+      <c r="V27" s="6"/>
+    </row>
+    <row r="28" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="X28" s="11"/>
+      <c r="Y28" s="11"/>
+    </row>
+    <row r="29" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="7">
+        <v>13</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="9">
+        <v>46237</v>
+      </c>
+      <c r="E29" s="9">
+        <v>46250</v>
+      </c>
+      <c r="F29" s="10">
+        <v>2</v>
+      </c>
+      <c r="G29" s="10">
+        <v>100</v>
+      </c>
+      <c r="H29" t="s">
+        <v>51</v>
+      </c>
+      <c r="W29" s="6"/>
+      <c r="X29" s="6"/>
+    </row>
+    <row r="30" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="7"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="Z30" s="11"/>
+    </row>
+    <row r="31" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="7">
+        <v>14</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="9">
+        <v>46251</v>
+      </c>
+      <c r="E31" s="9">
+        <v>46257</v>
+      </c>
+      <c r="F31" s="10">
+        <v>1</v>
+      </c>
+      <c r="G31" s="10">
+        <v>100</v>
+      </c>
+      <c r="H31" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y31" s="6"/>
+    </row>
+    <row r="32" spans="1:27" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="Z32" s="11"/>
+      <c r="AA32" s="11"/>
+    </row>
+    <row r="33" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="7">
+        <v>15</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="9">
+        <v>46258</v>
+      </c>
+      <c r="E33" s="9">
+        <v>46271</v>
+      </c>
+      <c r="F33" s="10">
+        <v>2</v>
+      </c>
+      <c r="G33" s="10">
+        <v>100</v>
+      </c>
+      <c r="H33" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z33" s="6"/>
+      <c r="AA33" s="6"/>
+    </row>
+    <row r="34" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="7"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="Z34" s="11"/>
+      <c r="AA34" s="11"/>
+      <c r="AB34" s="11"/>
+    </row>
+    <row r="35" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="7">
+        <v>16</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D35" s="9">
+        <v>46272</v>
+      </c>
+      <c r="E35" s="9">
+        <v>46278</v>
+      </c>
+      <c r="F35" s="10">
+        <v>1</v>
+      </c>
+      <c r="G35" s="10">
+        <v>100</v>
+      </c>
+      <c r="H35" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB35" s="12"/>
+    </row>
+    <row r="36" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="7"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="AB36" s="12"/>
+    </row>
+    <row r="37" spans="1:30" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="7">
+        <v>17</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37" s="9">
+        <v>46279</v>
+      </c>
+      <c r="E37" s="9">
+        <v>46285</v>
+      </c>
+      <c r="F37" s="10">
+        <v>1</v>
+      </c>
+      <c r="G37" s="10">
         <v>0</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H37" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC37" s="5"/>
+    </row>
+    <row r="38" spans="1:30" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="7"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="AC38" s="5"/>
+    </row>
+    <row r="39" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="7">
+        <v>18</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39" s="9">
+        <v>46286</v>
+      </c>
+      <c r="E39" s="9">
+        <v>46292</v>
+      </c>
+      <c r="F39" s="10">
+        <v>1</v>
+      </c>
+      <c r="G39" s="10">
+        <v>0</v>
+      </c>
+      <c r="H39" t="s">
         <v>32</v>
       </c>
-      <c r="AC19" s="5"/>
-    </row>
-    <row r="20" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="7">
-        <v>18</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="9">
-        <v>46286</v>
-      </c>
-      <c r="E20" s="9">
-        <v>46292</v>
-      </c>
-      <c r="F20" s="10">
-        <v>1</v>
-      </c>
-      <c r="G20" s="10">
-        <v>0</v>
-      </c>
-      <c r="H20" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD20" s="5"/>
+      <c r="AD39" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="Z1:AB1"/>
+    <mergeCell ref="U1:Y1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="L1:P1"/>
+    <mergeCell ref="I1:K1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>